<commit_message>
Task 3: Exploratory Testing - finished
</commit_message>
<xml_diff>
--- a/Exam/gymtrackerpro/__tests__/ft/proxy/proxy-ft-form.xlsx
+++ b/Exam/gymtrackerpro/__tests__/ft/proxy/proxy-ft-form.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="127" uniqueCount="78">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="118" uniqueCount="74">
   <si>
     <t>Component: proxy — proxy - protects admin and member routes by checking Iron Session authentication, role, and member active status before allowing or redirecting requests.</t>
   </si>
@@ -61,18 +61,6 @@
   </si>
   <si>
     <t>getIronSession(request, response, sessionOptions) is called for every request. Protected routes redirect to /login when unauthenticated and /unauthorized when role or active-status checks fail.</t>
-  </si>
-  <si>
-    <t>Remarks</t>
-  </si>
-  <si>
-    <t>Run: npx jest __tests__/ft/proxy/proxy.test.ts --selectProjects jsdom</t>
-  </si>
-  <si>
-    <t>Although proxy has no rendered DOM, it is included in FT because it protects frontend route access. NextResponse is mocked so the suite can run in the jsdom FT project.</t>
-  </si>
-  <si>
-    <t>Suite is kept in a single main describe block and covers matcher config plus every route/auth/role/active-status decision branch.</t>
   </si>
   <si>
     <t>No TC</t>
@@ -687,7 +675,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:B16"/>
+  <dimension ref="A1:B11"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
@@ -776,50 +764,11 @@
         <v>15</v>
       </c>
     </row>
-    <row r="12" ht="20" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A12" t="s">
-        <v>1</v>
-      </c>
-      <c r="B12" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="13" ht="20" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A13" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="B13" s="2"/>
-    </row>
-    <row r="14" ht="20" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A14" s="4" t="s">
-        <v>1</v>
-      </c>
-      <c r="B14" s="4" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="15" ht="50" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A15" s="4" t="s">
-        <v>1</v>
-      </c>
-      <c r="B15" s="4" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="16" ht="35" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A16" s="4" t="s">
-        <v>1</v>
-      </c>
-      <c r="B16" s="4" t="s">
-        <v>19</v>
-      </c>
-    </row>
   </sheetData>
-  <mergeCells count="4">
+  <mergeCells count="3">
     <mergeCell ref="A1:B1"/>
     <mergeCell ref="A3:B3"/>
     <mergeCell ref="A9:B9"/>
-    <mergeCell ref="A13:B13"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
@@ -844,22 +793,22 @@
         <v>1</v>
       </c>
       <c r="B1" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="C1" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="D1" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="E1" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="F1" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="C1" s="5" t="s">
+      <c r="G1" s="5" t="s">
         <v>21</v>
-      </c>
-      <c r="D1" s="5" t="s">
-        <v>22</v>
-      </c>
-      <c r="E1" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="F1" s="5" t="s">
-        <v>24</v>
-      </c>
-      <c r="G1" s="5" t="s">
-        <v>25</v>
       </c>
     </row>
     <row r="2" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
@@ -867,22 +816,22 @@
         <v>1</v>
       </c>
       <c r="B2" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="C2" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="D2" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="E2" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="F2" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="C2" s="4" t="s">
+      <c r="G2" s="7" t="s">
         <v>27</v>
-      </c>
-      <c r="D2" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="E2" s="4" t="s">
-        <v>29</v>
-      </c>
-      <c r="F2" s="4" t="s">
-        <v>30</v>
-      </c>
-      <c r="G2" s="7" t="s">
-        <v>31</v>
       </c>
     </row>
     <row r="3" ht="35" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
@@ -890,22 +839,22 @@
         <v>1</v>
       </c>
       <c r="B3" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="C3" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="D3" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="E3" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="F3" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="C3" s="4" t="s">
-        <v>33</v>
-      </c>
-      <c r="D3" s="4" t="s">
-        <v>34</v>
-      </c>
-      <c r="E3" s="4" t="s">
-        <v>35</v>
-      </c>
-      <c r="F3" s="4" t="s">
-        <v>36</v>
-      </c>
       <c r="G3" s="7" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
     </row>
     <row r="4" ht="35" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
@@ -913,22 +862,22 @@
         <v>1</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>37</v>
+        <v>33</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="G4" s="7" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
     </row>
     <row r="5" ht="35" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
@@ -936,22 +885,22 @@
         <v>1</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>42</v>
+        <v>38</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>43</v>
+        <v>39</v>
       </c>
       <c r="E5" s="4" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="F5" s="4" t="s">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="G5" s="7" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
     </row>
     <row r="6" ht="35" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
@@ -959,22 +908,22 @@
         <v>1</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
       <c r="E6" s="4" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="F6" s="4" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="G6" s="7" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
     </row>
     <row r="7" ht="35" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
@@ -982,22 +931,22 @@
         <v>1</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>50</v>
+        <v>46</v>
       </c>
       <c r="D7" s="4" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="E7" s="4" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="F7" s="4" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="G7" s="7" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
     </row>
     <row r="8" ht="35" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
@@ -1005,22 +954,22 @@
         <v>1</v>
       </c>
       <c r="B8" s="6" t="s">
-        <v>52</v>
+        <v>48</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
       <c r="E8" s="4" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="F8" s="4" t="s">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="G8" s="7" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
     </row>
     <row r="9" ht="35" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
@@ -1028,22 +977,22 @@
         <v>1</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>55</v>
+        <v>51</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>56</v>
+        <v>52</v>
       </c>
       <c r="D9" s="4" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="E9" s="4" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="F9" s="4" t="s">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="G9" s="7" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
     </row>
     <row r="10" ht="35" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
@@ -1051,22 +1000,22 @@
         <v>1</v>
       </c>
       <c r="B10" s="6" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>59</v>
+        <v>55</v>
       </c>
       <c r="D10" s="4" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="E10" s="4" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="F10" s="4" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="G10" s="7" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
     </row>
   </sheetData>
@@ -1094,17 +1043,17 @@
         <v>1</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>61</v>
+        <v>57</v>
       </c>
       <c r="D4" s="2"/>
       <c r="E4" s="2"/>
       <c r="F4" s="2"/>
       <c r="G4" s="2"/>
       <c r="H4" s="2" t="s">
-        <v>62</v>
+        <v>58</v>
       </c>
       <c r="I4" s="2" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="J4" s="2"/>
       <c r="K4" s="2"/>
@@ -1116,40 +1065,40 @@
         <v>1</v>
       </c>
       <c r="B5" s="5" t="s">
+        <v>60</v>
+      </c>
+      <c r="C5" s="5" t="s">
+        <v>61</v>
+      </c>
+      <c r="D5" s="5" t="s">
+        <v>62</v>
+      </c>
+      <c r="E5" s="5" t="s">
+        <v>63</v>
+      </c>
+      <c r="F5" s="5" t="s">
         <v>64</v>
       </c>
-      <c r="C5" s="5" t="s">
+      <c r="G5" s="5" t="s">
         <v>65</v>
       </c>
-      <c r="D5" s="5" t="s">
+      <c r="H5" s="5" t="s">
         <v>66</v>
       </c>
-      <c r="E5" s="5" t="s">
+      <c r="I5" s="5" t="s">
         <v>67</v>
       </c>
-      <c r="F5" s="5" t="s">
-        <v>68</v>
-      </c>
-      <c r="G5" s="5" t="s">
-        <v>69</v>
-      </c>
-      <c r="H5" s="5" t="s">
-        <v>70</v>
-      </c>
-      <c r="I5" s="5" t="s">
-        <v>71</v>
-      </c>
       <c r="J5" s="5" t="s">
-        <v>65</v>
+        <v>61</v>
       </c>
       <c r="K5" s="5" t="s">
-        <v>66</v>
+        <v>62</v>
       </c>
       <c r="L5" s="5" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
       <c r="M5" s="5" t="s">
-        <v>68</v>
+        <v>64</v>
       </c>
     </row>
     <row r="6" ht="20" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
@@ -1157,7 +1106,7 @@
         <v>1</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>72</v>
+        <v>68</v>
       </c>
       <c r="C6" s="4">
         <v>9</v>
@@ -1169,28 +1118,28 @@
         <v>0</v>
       </c>
       <c r="F6" s="4" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="G6" s="4">
         <v>0</v>
       </c>
       <c r="H6" s="4" t="s">
-        <v>74</v>
+        <v>70</v>
       </c>
       <c r="I6" s="4" t="s">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="J6" s="4">
         <v>0</v>
       </c>
       <c r="K6" s="4" t="s">
-        <v>76</v>
+        <v>72</v>
       </c>
       <c r="L6" s="4" t="s">
-        <v>76</v>
+        <v>72</v>
       </c>
       <c r="M6" s="4" t="s">
-        <v>76</v>
+        <v>72</v>
       </c>
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.25"/>
@@ -1199,7 +1148,7 @@
         <v>1</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>77</v>
+        <v>73</v>
       </c>
       <c r="C8" s="4" t="s">
         <v>4</v>

</xml_diff>